<commit_message>
testing new format page
</commit_message>
<xml_diff>
--- a/pipeline/source/geoschool-2026/Codebook-geoschool-2026.xlsx
+++ b/pipeline/source/geoschool-2026/Codebook-geoschool-2026.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dependencia administrativa normalizada: Publico, Subvencionado o Privado. CL: COD_DEPE; CO: prestador_de_servicio; PE: GES_DEP.</t>
+          <t>Dependencia administrativa normalizada: Publico, Subvencionado o Privado. CL: COD_DEPE; CO: SECTOR (SISE-DANE); PE: GES_DEP.</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Directorio de Establecimientos Educativos (datos.gov.co / Socrata).</t>
+          <t>DANE SISE — Sedes Educativas georreferenciadas (Activas).</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INPUT/Extraction-*-CO/*.csv (generado por 01-Extraction/extract_co.py).</t>
+          <t>INPUT/Extraction-*-CO/SEDES_EDUCATIVAS_SISE-COLOMBIA.csv.</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Join con capa DANE SISE (MapaAnalisisEspacialCDGE) por código DANE.</t>
+          <t>Coordenadas incluidas en la extracción (LATITUD/LONGITUD).</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Derivado de prestador_de_servicio (OFICIAL → Publico; resto → Privado).</t>
+          <t>Derivado de SECTOR (OFICIAL → Publico; NO OFICIAL → Privado).</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Un registro por establecimiento (código DANE).</t>
+          <t>Un registro por sede educativa (COD_DANE).</t>
         </is>
       </c>
     </row>

</xml_diff>